<commit_message>
New Exam Portal redesigned
</commit_message>
<xml_diff>
--- a/RESULTS/2017/CLASS/SS1/Chemistry/results.xlsx
+++ b/RESULTS/2017/CLASS/SS1/Chemistry/results.xlsx
@@ -413,9 +413,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Admission No</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Score (%)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Time Taken</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Submitted At</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>